<commit_message>
Update MLB weather 2026-07-20 09:41 AM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v5_2026_07_20.xlsx
+++ b/mlb_weather_professional_v5_2026_07_20.xlsx
@@ -614,49 +614,49 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-20 09:38:04 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:06 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:10 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:11 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:13 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:14 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:15 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:16 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:17 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:19 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:20 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:22 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:23 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:24 AM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-20 09:38:25 AM PDT</t>
+    <t>2026-07-20 09:41:20 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:21 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:22 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:23 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:25 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:26 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:27 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:28 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:29 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:30 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:31 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:32 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:33 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:34 AM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-20 09:41:35 AM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -1064,49 +1064,49 @@
     <t>10:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-20 16:38:04 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:06 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:10 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:11 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:13 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:14 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:15 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:16 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:17 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:19 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:20 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:22 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:23 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:24 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-20 16:38:25 UTC</t>
+    <t>2026-07-20 16:41:20 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:21 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:22 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:23 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:25 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:26 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:27 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:28 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:29 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:30 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:31 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:32 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:33 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:34 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-20 16:41:35 UTC</t>
   </si>
   <si>
     <t>2026-07-20T07:46:59+00:00</t>
@@ -1927,22 +1927,22 @@
         <v>150</v>
       </c>
       <c r="N2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="O2" t="s">
         <v>159</v>
       </c>
       <c r="P2">
-        <v>-1.4</v>
+        <v>-1.3</v>
       </c>
       <c r="Q2">
         <v>-1</v>
       </c>
       <c r="R2">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="S2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="U2" t="s">
         <v>167</v>
@@ -2014,7 +2014,7 @@
         <v>189</v>
       </c>
       <c r="AR2">
-        <v>-0.7</v>
+        <v>-1</v>
       </c>
       <c r="AS2">
         <v>0</v>
@@ -2038,7 +2038,7 @@
         <v>197</v>
       </c>
       <c r="AZ2">
-        <v>531.1</v>
+        <v>534.4</v>
       </c>
       <c r="BA2">
         <v>5</v>
@@ -2172,7 +2172,7 @@
         <v>189</v>
       </c>
       <c r="AR3">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="AS3">
         <v>0</v>
@@ -2196,7 +2196,7 @@
         <v>198</v>
       </c>
       <c r="AZ3">
-        <v>630.1</v>
+        <v>633.4</v>
       </c>
       <c r="BA3">
         <v>5</v>
@@ -2330,7 +2330,7 @@
         <v>190</v>
       </c>
       <c r="AR4">
-        <v>11.8</v>
+        <v>7.8</v>
       </c>
       <c r="AS4">
         <v>0</v>
@@ -2488,7 +2488,7 @@
         <v>190</v>
       </c>
       <c r="AR5">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="AS5">
         <v>0</v>
@@ -2512,7 +2512,7 @@
         <v>200</v>
       </c>
       <c r="AZ5">
-        <v>41.2</v>
+        <v>44.4</v>
       </c>
       <c r="BA5">
         <v>5</v>
@@ -2646,7 +2646,7 @@
         <v>190</v>
       </c>
       <c r="AR6">
-        <v>7.1</v>
+        <v>6.2</v>
       </c>
       <c r="AS6">
         <v>0</v>
@@ -2670,7 +2670,7 @@
         <v>201</v>
       </c>
       <c r="AZ6">
-        <v>510.2</v>
+        <v>513.4</v>
       </c>
       <c r="BA6">
         <v>5</v>
@@ -2804,7 +2804,7 @@
         <v>191</v>
       </c>
       <c r="AR7">
-        <v>-1.6</v>
+        <v>-1.5</v>
       </c>
       <c r="AS7">
         <v>0</v>
@@ -2828,7 +2828,7 @@
         <v>202</v>
       </c>
       <c r="AZ7">
-        <v>10.9</v>
+        <v>14.1</v>
       </c>
       <c r="BA7">
         <v>5</v>
@@ -2962,7 +2962,7 @@
         <v>190</v>
       </c>
       <c r="AR8">
-        <v>5.7</v>
+        <v>4.7</v>
       </c>
       <c r="AS8">
         <v>0</v>
@@ -2986,7 +2986,7 @@
         <v>203</v>
       </c>
       <c r="AZ8">
-        <v>25.4</v>
+        <v>28.6</v>
       </c>
       <c r="BA8">
         <v>5</v>
@@ -3144,7 +3144,7 @@
         <v>204</v>
       </c>
       <c r="AZ9">
-        <v>64.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="BA9">
         <v>5</v>
@@ -3278,7 +3278,7 @@
         <v>190</v>
       </c>
       <c r="AR10">
-        <v>13.6</v>
+        <v>15.2</v>
       </c>
       <c r="AS10">
         <v>0</v>
@@ -3296,13 +3296,13 @@
         <v>193</v>
       </c>
       <c r="AX10">
-        <v>14.8</v>
+        <v>14.7</v>
       </c>
       <c r="AY10" t="s">
         <v>205</v>
       </c>
       <c r="AZ10">
-        <v>42.3</v>
+        <v>45.5</v>
       </c>
       <c r="BA10">
         <v>5</v>
@@ -3460,7 +3460,7 @@
         <v>206</v>
       </c>
       <c r="AZ11">
-        <v>41.3</v>
+        <v>44.5</v>
       </c>
       <c r="BA11">
         <v>5</v>
@@ -3612,13 +3612,13 @@
         <v>196</v>
       </c>
       <c r="AX12">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="AY12" t="s">
         <v>207</v>
       </c>
       <c r="AZ12">
-        <v>85.8</v>
+        <v>89</v>
       </c>
       <c r="BA12">
         <v>5</v>
@@ -3749,10 +3749,10 @@
         <v>19.9</v>
       </c>
       <c r="AQ13" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AR13">
-        <v>-0.7</v>
+        <v>2.3</v>
       </c>
       <c r="AS13">
         <v>0</v>
@@ -3776,7 +3776,7 @@
         <v>208</v>
       </c>
       <c r="AZ13">
-        <v>447.1</v>
+        <v>450.3</v>
       </c>
       <c r="BA13">
         <v>5</v>
@@ -3934,7 +3934,7 @@
         <v>209</v>
       </c>
       <c r="AZ14">
-        <v>285.4</v>
+        <v>288.6</v>
       </c>
       <c r="BA14">
         <v>5</v>
@@ -4068,7 +4068,7 @@
         <v>189</v>
       </c>
       <c r="AR15">
-        <v>-0.4</v>
+        <v>-0.9</v>
       </c>
       <c r="AS15">
         <v>0</v>
@@ -4092,7 +4092,7 @@
         <v>210</v>
       </c>
       <c r="AZ15">
-        <v>612.2</v>
+        <v>615.4</v>
       </c>
       <c r="BA15">
         <v>5</v>
@@ -4226,7 +4226,7 @@
         <v>190</v>
       </c>
       <c r="AR16">
-        <v>4.6</v>
+        <v>4.2</v>
       </c>
       <c r="AS16">
         <v>0</v>
@@ -4250,7 +4250,7 @@
         <v>211</v>
       </c>
       <c r="AZ16">
-        <v>530.6</v>
+        <v>533.8</v>
       </c>
       <c r="BA16">
         <v>5</v>
@@ -4719,7 +4719,7 @@
         <v>362</v>
       </c>
       <c r="J2">
-        <v>531.1</v>
+        <v>534.4</v>
       </c>
       <c r="K2">
         <v>6</v>
@@ -4767,7 +4767,7 @@
         <v>94.90000000000001</v>
       </c>
       <c r="Z2">
-        <v>55</v>
+        <v>54.9</v>
       </c>
       <c r="AA2">
         <v>0.92</v>
@@ -4818,13 +4818,13 @@
         <v>1</v>
       </c>
       <c r="AQ2">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="AR2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="AS2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="AT2">
         <v>8.800000000000001</v>
@@ -4836,13 +4836,13 @@
         <v>8.1</v>
       </c>
       <c r="AW2">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="AX2" t="s">
         <v>159</v>
       </c>
       <c r="AY2">
-        <v>311.8</v>
+        <v>315.4</v>
       </c>
       <c r="AZ2" t="s">
         <v>393</v>
@@ -4851,61 +4851,61 @@
         <v>393</v>
       </c>
       <c r="BB2">
-        <v>23.5</v>
+        <v>22</v>
       </c>
       <c r="BC2">
-        <v>23.5</v>
+        <v>22</v>
       </c>
       <c r="BD2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="BE2">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="BF2">
-        <v>27.5</v>
+        <v>30.8</v>
       </c>
       <c r="BG2">
+        <v>-1.3</v>
+      </c>
+      <c r="BH2">
+        <v>-1.7</v>
+      </c>
+      <c r="BI2">
+        <v>-0.3</v>
+      </c>
+      <c r="BJ2">
+        <v>1.2</v>
+      </c>
+      <c r="BK2">
         <v>-1.2</v>
-      </c>
-      <c r="BH2">
-        <v>-1.8</v>
-      </c>
-      <c r="BI2">
-        <v>-0.2</v>
-      </c>
-      <c r="BJ2">
-        <v>1.3</v>
-      </c>
-      <c r="BK2">
-        <v>-1.1</v>
       </c>
       <c r="BL2">
         <v>-1.6</v>
       </c>
       <c r="BM2">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="BN2">
-        <v>-1.2</v>
+        <v>-1.3</v>
       </c>
       <c r="BO2">
-        <v>-1.8</v>
+        <v>-1.7</v>
       </c>
       <c r="BP2">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="BQ2">
         <v>-1</v>
       </c>
       <c r="BR2">
-        <v>-1.4</v>
+        <v>-1.3</v>
       </c>
       <c r="BS2">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="BT2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="BU2">
         <v>-0.9</v>
@@ -4947,13 +4947,13 @@
         <v>139</v>
       </c>
       <c r="CH2">
-        <v>55.2</v>
+        <v>55.1</v>
       </c>
       <c r="CI2">
         <v>7.7</v>
       </c>
       <c r="CJ2">
-        <v>-2.7</v>
+        <v>-2.8</v>
       </c>
       <c r="CK2">
         <v>0</v>
@@ -4962,16 +4962,16 @@
         <v>0</v>
       </c>
       <c r="CM2">
-        <v>1.013</v>
+        <v>1.012</v>
       </c>
       <c r="CN2">
-        <v>55.9</v>
+        <v>55.7</v>
       </c>
       <c r="CO2">
         <v>54.8</v>
       </c>
       <c r="CP2">
-        <v>54.2</v>
+        <v>54.1</v>
       </c>
       <c r="CQ2">
         <v>51.4</v>
@@ -5033,7 +5033,7 @@
         <v>362</v>
       </c>
       <c r="J3">
-        <v>531.1</v>
+        <v>534.4</v>
       </c>
       <c r="K3">
         <v>7</v>
@@ -5347,7 +5347,7 @@
         <v>362</v>
       </c>
       <c r="J4">
-        <v>531.1</v>
+        <v>534.4</v>
       </c>
       <c r="K4">
         <v>8</v>
@@ -5661,7 +5661,7 @@
         <v>362</v>
       </c>
       <c r="J5">
-        <v>531.1</v>
+        <v>534.4</v>
       </c>
       <c r="K5">
         <v>9</v>
@@ -5975,7 +5975,7 @@
         <v>363</v>
       </c>
       <c r="J6">
-        <v>630.1</v>
+        <v>633.4</v>
       </c>
       <c r="K6">
         <v>6.4</v>
@@ -6289,7 +6289,7 @@
         <v>363</v>
       </c>
       <c r="J7">
-        <v>630.1</v>
+        <v>633.4</v>
       </c>
       <c r="K7">
         <v>7.4</v>
@@ -6603,7 +6603,7 @@
         <v>363</v>
       </c>
       <c r="J8">
-        <v>630.1</v>
+        <v>633.4</v>
       </c>
       <c r="K8">
         <v>8.4</v>
@@ -6917,7 +6917,7 @@
         <v>363</v>
       </c>
       <c r="J9">
-        <v>630.1</v>
+        <v>633.4</v>
       </c>
       <c r="K9">
         <v>9.4</v>
@@ -7231,7 +7231,7 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="L10">
         <v>4</v>
@@ -7539,7 +7539,7 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="L11">
         <v>4</v>
@@ -7847,7 +7847,7 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="L12">
         <v>4</v>
@@ -8155,7 +8155,7 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="L13">
         <v>4</v>
@@ -8463,7 +8463,7 @@
         <v>364</v>
       </c>
       <c r="J14">
-        <v>41.2</v>
+        <v>44.4</v>
       </c>
       <c r="K14">
         <v>6.5</v>
@@ -8508,7 +8508,7 @@
         <v>19.7</v>
       </c>
       <c r="Y14">
-        <v>88.59999999999999</v>
+        <v>88.7</v>
       </c>
       <c r="Z14">
         <v>66.2</v>
@@ -8777,7 +8777,7 @@
         <v>364</v>
       </c>
       <c r="J15">
-        <v>41.2</v>
+        <v>44.4</v>
       </c>
       <c r="K15">
         <v>7.5</v>
@@ -9091,7 +9091,7 @@
         <v>364</v>
       </c>
       <c r="J16">
-        <v>41.2</v>
+        <v>44.4</v>
       </c>
       <c r="K16">
         <v>8.5</v>
@@ -9405,7 +9405,7 @@
         <v>364</v>
       </c>
       <c r="J17">
-        <v>41.2</v>
+        <v>44.4</v>
       </c>
       <c r="K17">
         <v>9.5</v>
@@ -9719,7 +9719,7 @@
         <v>365</v>
       </c>
       <c r="J18">
-        <v>510.2</v>
+        <v>513.4</v>
       </c>
       <c r="K18">
         <v>6.5</v>
@@ -10033,7 +10033,7 @@
         <v>365</v>
       </c>
       <c r="J19">
-        <v>510.2</v>
+        <v>513.4</v>
       </c>
       <c r="K19">
         <v>7.5</v>
@@ -10347,7 +10347,7 @@
         <v>365</v>
       </c>
       <c r="J20">
-        <v>510.2</v>
+        <v>513.4</v>
       </c>
       <c r="K20">
         <v>8.5</v>
@@ -10661,7 +10661,7 @@
         <v>365</v>
       </c>
       <c r="J21">
-        <v>510.2</v>
+        <v>513.4</v>
       </c>
       <c r="K21">
         <v>9.5</v>
@@ -10975,7 +10975,7 @@
         <v>366</v>
       </c>
       <c r="J22">
-        <v>10.9</v>
+        <v>14.1</v>
       </c>
       <c r="K22">
         <v>6.6</v>
@@ -11289,7 +11289,7 @@
         <v>366</v>
       </c>
       <c r="J23">
-        <v>10.9</v>
+        <v>14.1</v>
       </c>
       <c r="K23">
         <v>7.6</v>
@@ -11603,7 +11603,7 @@
         <v>366</v>
       </c>
       <c r="J24">
-        <v>10.9</v>
+        <v>14.1</v>
       </c>
       <c r="K24">
         <v>8.6</v>
@@ -11917,7 +11917,7 @@
         <v>366</v>
       </c>
       <c r="J25">
-        <v>10.9</v>
+        <v>14.1</v>
       </c>
       <c r="K25">
         <v>9.6</v>
@@ -12231,7 +12231,7 @@
         <v>367</v>
       </c>
       <c r="J26">
-        <v>25.4</v>
+        <v>28.6</v>
       </c>
       <c r="K26">
         <v>7</v>
@@ -12545,7 +12545,7 @@
         <v>367</v>
       </c>
       <c r="J27">
-        <v>25.4</v>
+        <v>28.6</v>
       </c>
       <c r="K27">
         <v>8</v>
@@ -12859,7 +12859,7 @@
         <v>367</v>
       </c>
       <c r="J28">
-        <v>25.4</v>
+        <v>28.6</v>
       </c>
       <c r="K28">
         <v>9</v>
@@ -12904,7 +12904,7 @@
         <v>12.2</v>
       </c>
       <c r="Y28">
-        <v>90.7</v>
+        <v>90.8</v>
       </c>
       <c r="Z28">
         <v>72.7</v>
@@ -13173,7 +13173,7 @@
         <v>367</v>
       </c>
       <c r="J29">
-        <v>25.4</v>
+        <v>28.6</v>
       </c>
       <c r="K29">
         <v>10</v>
@@ -13487,7 +13487,7 @@
         <v>368</v>
       </c>
       <c r="J30">
-        <v>64.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K30">
         <v>7</v>
@@ -13801,7 +13801,7 @@
         <v>368</v>
       </c>
       <c r="J31">
-        <v>64.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K31">
         <v>8</v>
@@ -14115,7 +14115,7 @@
         <v>368</v>
       </c>
       <c r="J32">
-        <v>64.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K32">
         <v>9</v>
@@ -14429,7 +14429,7 @@
         <v>368</v>
       </c>
       <c r="J33">
-        <v>64.7</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K33">
         <v>10</v>
@@ -14743,7 +14743,7 @@
         <v>369</v>
       </c>
       <c r="J34">
-        <v>42.3</v>
+        <v>45.5</v>
       </c>
       <c r="K34">
         <v>7.4</v>
@@ -15057,7 +15057,7 @@
         <v>369</v>
       </c>
       <c r="J35">
-        <v>42.3</v>
+        <v>45.5</v>
       </c>
       <c r="K35">
         <v>8.4</v>
@@ -15371,7 +15371,7 @@
         <v>369</v>
       </c>
       <c r="J36">
-        <v>42.3</v>
+        <v>45.5</v>
       </c>
       <c r="K36">
         <v>9.4</v>
@@ -15685,7 +15685,7 @@
         <v>369</v>
       </c>
       <c r="J37">
-        <v>42.3</v>
+        <v>45.5</v>
       </c>
       <c r="K37">
         <v>10.4</v>
@@ -15952,7 +15952,7 @@
         <v>195</v>
       </c>
       <c r="CU37">
-        <v>14.8</v>
+        <v>14.7</v>
       </c>
       <c r="CV37" t="s">
         <v>193</v>
@@ -15999,7 +15999,7 @@
         <v>370</v>
       </c>
       <c r="J38">
-        <v>41.3</v>
+        <v>44.5</v>
       </c>
       <c r="K38">
         <v>7.4</v>
@@ -16313,7 +16313,7 @@
         <v>370</v>
       </c>
       <c r="J39">
-        <v>41.3</v>
+        <v>44.5</v>
       </c>
       <c r="K39">
         <v>8.4</v>
@@ -16627,7 +16627,7 @@
         <v>370</v>
       </c>
       <c r="J40">
-        <v>41.3</v>
+        <v>44.5</v>
       </c>
       <c r="K40">
         <v>9.4</v>
@@ -16941,7 +16941,7 @@
         <v>370</v>
       </c>
       <c r="J41">
-        <v>41.3</v>
+        <v>44.5</v>
       </c>
       <c r="K41">
         <v>10.4</v>
@@ -17255,7 +17255,7 @@
         <v>371</v>
       </c>
       <c r="J42">
-        <v>85.8</v>
+        <v>89</v>
       </c>
       <c r="K42">
         <v>7.5</v>
@@ -17569,7 +17569,7 @@
         <v>371</v>
       </c>
       <c r="J43">
-        <v>85.8</v>
+        <v>89</v>
       </c>
       <c r="K43">
         <v>8.5</v>
@@ -17836,7 +17836,7 @@
         <v>194</v>
       </c>
       <c r="CU43">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="CV43" t="s">
         <v>196</v>
@@ -17883,7 +17883,7 @@
         <v>371</v>
       </c>
       <c r="J44">
-        <v>85.8</v>
+        <v>89</v>
       </c>
       <c r="K44">
         <v>9.5</v>
@@ -18197,7 +18197,7 @@
         <v>371</v>
       </c>
       <c r="J45">
-        <v>85.8</v>
+        <v>89</v>
       </c>
       <c r="K45">
         <v>10.5</v>
@@ -18464,7 +18464,7 @@
         <v>194</v>
       </c>
       <c r="CU45">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="CV45" t="s">
         <v>193</v>
@@ -18511,7 +18511,7 @@
         <v>372</v>
       </c>
       <c r="J46">
-        <v>447.1</v>
+        <v>450.3</v>
       </c>
       <c r="K46">
         <v>8</v>
@@ -18825,7 +18825,7 @@
         <v>372</v>
       </c>
       <c r="J47">
-        <v>447.1</v>
+        <v>450.3</v>
       </c>
       <c r="K47">
         <v>9</v>
@@ -19139,7 +19139,7 @@
         <v>372</v>
       </c>
       <c r="J48">
-        <v>447.1</v>
+        <v>450.3</v>
       </c>
       <c r="K48">
         <v>10</v>
@@ -19453,7 +19453,7 @@
         <v>372</v>
       </c>
       <c r="J49">
-        <v>447.1</v>
+        <v>450.3</v>
       </c>
       <c r="K49">
         <v>11</v>
@@ -19767,7 +19767,7 @@
         <v>373</v>
       </c>
       <c r="J50">
-        <v>285.4</v>
+        <v>288.6</v>
       </c>
       <c r="K50">
         <v>9</v>
@@ -20081,7 +20081,7 @@
         <v>373</v>
       </c>
       <c r="J51">
-        <v>285.4</v>
+        <v>288.6</v>
       </c>
       <c r="K51">
         <v>10</v>
@@ -20395,7 +20395,7 @@
         <v>373</v>
       </c>
       <c r="J52">
-        <v>285.4</v>
+        <v>288.6</v>
       </c>
       <c r="K52">
         <v>11</v>
@@ -20709,7 +20709,7 @@
         <v>373</v>
       </c>
       <c r="J53">
-        <v>285.4</v>
+        <v>288.6</v>
       </c>
       <c r="K53">
         <v>12</v>
@@ -20808,7 +20808,7 @@
         <v>510</v>
       </c>
       <c r="AQ53">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
       <c r="AR53">
         <v>0</v>
@@ -20829,10 +20829,10 @@
         <v>0</v>
       </c>
       <c r="AX53" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="AY53">
-        <v>253.6</v>
+        <v>258.8</v>
       </c>
       <c r="AZ53" t="s">
         <v>398</v>
@@ -20841,19 +20841,19 @@
         <v>398</v>
       </c>
       <c r="BB53">
-        <v>70.3</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="BC53">
-        <v>70.3</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="BD53">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="BE53">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="BF53">
-        <v>35.9</v>
+        <v>40.8</v>
       </c>
       <c r="BG53">
         <v>0</v>
@@ -21023,7 +21023,7 @@
         <v>374</v>
       </c>
       <c r="J54">
-        <v>612.2</v>
+        <v>615.4</v>
       </c>
       <c r="K54">
         <v>9</v>
@@ -21337,7 +21337,7 @@
         <v>374</v>
       </c>
       <c r="J55">
-        <v>612.2</v>
+        <v>615.4</v>
       </c>
       <c r="K55">
         <v>10</v>
@@ -21651,7 +21651,7 @@
         <v>374</v>
       </c>
       <c r="J56">
-        <v>612.2</v>
+        <v>615.4</v>
       </c>
       <c r="K56">
         <v>11</v>
@@ -21965,7 +21965,7 @@
         <v>374</v>
       </c>
       <c r="J57">
-        <v>612.2</v>
+        <v>615.4</v>
       </c>
       <c r="K57">
         <v>12</v>
@@ -22064,13 +22064,13 @@
         <v>0</v>
       </c>
       <c r="AQ57">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="AR57">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="AS57">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="AT57">
         <v>7.1</v>
@@ -22082,13 +22082,13 @@
         <v>5.1</v>
       </c>
       <c r="AW57">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="AX57" t="s">
         <v>392</v>
       </c>
       <c r="AY57">
-        <v>352.2</v>
+        <v>351.5</v>
       </c>
       <c r="AZ57" t="s">
         <v>398</v>
@@ -22097,25 +22097,25 @@
         <v>398</v>
       </c>
       <c r="BB57">
-        <v>82.8</v>
+        <v>82.7</v>
       </c>
       <c r="BC57">
-        <v>82.8</v>
+        <v>82.7</v>
       </c>
       <c r="BD57">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="BE57">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="BF57">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="BG57">
-        <v>-1.6</v>
+        <v>-1.5</v>
       </c>
       <c r="BH57">
-        <v>-2.7</v>
+        <v>-2.6</v>
       </c>
       <c r="BI57">
         <v>0.1</v>
@@ -22133,25 +22133,25 @@
         <v>0.1</v>
       </c>
       <c r="BN57">
-        <v>-1.6</v>
+        <v>-1.5</v>
       </c>
       <c r="BO57">
-        <v>-2.7</v>
+        <v>-2.6</v>
       </c>
       <c r="BP57">
         <v>0.1</v>
       </c>
       <c r="BQ57">
-        <v>-0.9</v>
+        <v>-0.8</v>
       </c>
       <c r="BR57">
-        <v>-1.4</v>
+        <v>-1.3</v>
       </c>
       <c r="BS57">
         <v>0.1</v>
       </c>
       <c r="BT57">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="BU57">
         <v>-0.3</v>
@@ -22193,7 +22193,7 @@
         <v>143</v>
       </c>
       <c r="CH57">
-        <v>51.4</v>
+        <v>51.5</v>
       </c>
       <c r="CI57">
         <v>3.9</v>
@@ -22208,13 +22208,13 @@
         <v>0</v>
       </c>
       <c r="CM57">
-        <v>1.003</v>
+        <v>1.004</v>
       </c>
       <c r="CN57">
-        <v>51.7</v>
+        <v>51.8</v>
       </c>
       <c r="CO57">
-        <v>50.4</v>
+        <v>50.5</v>
       </c>
       <c r="CP57">
         <v>52.3</v>
@@ -22279,7 +22279,7 @@
         <v>375</v>
       </c>
       <c r="J58">
-        <v>530.6</v>
+        <v>533.8</v>
       </c>
       <c r="K58">
         <v>9.5</v>
@@ -22593,7 +22593,7 @@
         <v>375</v>
       </c>
       <c r="J59">
-        <v>530.6</v>
+        <v>533.8</v>
       </c>
       <c r="K59">
         <v>10.5</v>
@@ -22907,7 +22907,7 @@
         <v>375</v>
       </c>
       <c r="J60">
-        <v>530.6</v>
+        <v>533.8</v>
       </c>
       <c r="K60">
         <v>11.5</v>
@@ -23221,7 +23221,7 @@
         <v>375</v>
       </c>
       <c r="J61">
-        <v>530.6</v>
+        <v>533.8</v>
       </c>
       <c r="K61">
         <v>12.5</v>

</xml_diff>